<commit_message>
Add RSS auto-discovery and populate first item
</commit_message>
<xml_diff>
--- a/source.xlsx
+++ b/source.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="25">
   <si>
     <t>Course Title</t>
   </si>
@@ -83,6 +83,9 @@
   </si>
   <si>
     <t>https://www.udemy.com/course/aws-certified-devops-pro-mock-test/?referralCode=3781FAE259E0E89C23A7</t>
+  </si>
+  <si>
+    <t>done</t>
   </si>
   <si>
     <t>Pending</t>
@@ -489,7 +492,7 @@
         <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -500,7 +503,7 @@
         <v>15</v>
       </c>
       <c r="C4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -511,7 +514,7 @@
         <v>16</v>
       </c>
       <c r="C5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -522,7 +525,7 @@
         <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -533,7 +536,7 @@
         <v>18</v>
       </c>
       <c r="C7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -544,7 +547,7 @@
         <v>19</v>
       </c>
       <c r="C8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -555,7 +558,7 @@
         <v>20</v>
       </c>
       <c r="C9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -566,7 +569,7 @@
         <v>21</v>
       </c>
       <c r="C10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -577,7 +580,7 @@
         <v>22</v>
       </c>
       <c r="C11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>